<commit_message>
research: portfolio 20261026T152031546516Z-5f77f1ad [SUCCESS]
Imported from local commit: ce29750eaf170e55eca6c66eaff0267930427f80
Original author: Investment Workspace <workspace@localhost> (2026-10-26T15:20:31Z)
File tree preserved exactly from the uploaded Git bundle.
</commit_message>
<xml_diff>
--- a/workbooks/Investment_Workspace.xlsx
+++ b/workbooks/Investment_Workspace.xlsx
@@ -21,26 +21,32 @@
     <sheet name="Notes" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Assumptions" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Manual_Inputs" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Dividend_Calendar" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Earnings_Bridge" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Valuation" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Earnings_Bridge" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Entry_Levels" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Watchlist" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Catalysts" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="RS_Trend" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Sector_Rotation" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Mean_Reversion" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Macro" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Scenarios" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Portfolio_Risk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="IC_Actions" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Retirement" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Cross_Asset" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Entry_Levels" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Dividend_Calendar" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Top_10" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Watchlist" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Catalysts" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="RS_Trend" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Sector_Rotation" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Mean_Reversion" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Macro" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Scenarios" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Portfolio_Risk" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="IC_Actions" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Retirement" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Cross_Asset" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reconciliation'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Notes'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Manual_Inputs'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Earnings_Bridge'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Valuation'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Entry_Levels'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Dividend_Calendar'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Top_10'!$A$1:$B$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -188,8 +194,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:I3" headerRowCount="1">
-  <autoFilter ref="A1:I3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:I4" headerRowCount="1">
+  <autoFilter ref="A1:I4"/>
   <tableColumns count="9">
     <tableColumn id="1" name="cached_input_tokens"/>
     <tableColumn id="2" name="calculation_runtime_seconds"/>
@@ -223,7 +229,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T_Dividend_Calendar" displayName="T_Dividend_Calendar" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T_Watchlist" displayName="T_Watchlist" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -234,7 +240,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T_Valuation" displayName="T_Valuation" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T_Catalysts" displayName="T_Catalysts" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -245,7 +251,7 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="T_Earnings_Bridge" displayName="T_Earnings_Bridge" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="T_RS_Trend" displayName="T_RS_Trend" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -256,7 +262,7 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="T_Entry_Levels" displayName="T_Entry_Levels" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="T_Sector_Rotation" displayName="T_Sector_Rotation" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -267,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="T_Watchlist" displayName="T_Watchlist" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="T_Mean_Reversion" displayName="T_Mean_Reversion" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -278,7 +284,7 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="T_Catalysts" displayName="T_Catalysts" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="T_Macro" displayName="T_Macro" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -289,7 +295,7 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="T_RS_Trend" displayName="T_RS_Trend" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="T_Scenarios" displayName="T_Scenarios" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -300,7 +306,7 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="T_Sector_Rotation" displayName="T_Sector_Rotation" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="T_Portfolio_Risk" displayName="T_Portfolio_Risk" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -337,7 +343,7 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="T_Mean_Reversion" displayName="T_Mean_Reversion" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="T_IC_Actions" displayName="T_IC_Actions" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -348,7 +354,7 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="T_Macro" displayName="T_Macro" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="T_Retirement" displayName="T_Retirement" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -359,51 +365,7 @@
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="T_Scenarios" displayName="T_Scenarios" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="T_Portfolio_Risk" displayName="T_Portfolio_Risk" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="T_IC_Actions" displayName="T_IC_Actions" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="T_Retirement" displayName="T_Retirement" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="T_Cross_Asset" displayName="T_Cross_Asset" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="T_Cross_Asset" displayName="T_Cross_Asset" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -486,23 +448,23 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T_Coverage" displayName="T_Coverage" ref="A1:Q5" headerRowCount="1">
   <autoFilter ref="A1:Q5"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="assumption_ids"/>
-    <tableColumn id="2" name="code_version"/>
-    <tableColumn id="3" name="confidence"/>
-    <tableColumn id="4" name="effective_date"/>
-    <tableColumn id="5" name="input_hash"/>
-    <tableColumn id="6" name="market_cutoff_metadata"/>
-    <tableColumn id="7" name="outcome"/>
-    <tableColumn id="8" name="owner"/>
-    <tableColumn id="9" name="reason"/>
-    <tableColumn id="10" name="record_id"/>
-    <tableColumn id="11" name="run_id"/>
-    <tableColumn id="12" name="schema_version"/>
-    <tableColumn id="13" name="source_ids"/>
-    <tableColumn id="14" name="ticker"/>
-    <tableColumn id="15" name="units"/>
-    <tableColumn id="16" name="upstream_run_ids"/>
-    <tableColumn id="17" name="validation_status"/>
+    <tableColumn id="1" name="ticker"/>
+    <tableColumn id="2" name="outcome"/>
+    <tableColumn id="3" name="owner"/>
+    <tableColumn id="4" name="reason"/>
+    <tableColumn id="5" name="schema_version"/>
+    <tableColumn id="6" name="run_id"/>
+    <tableColumn id="7" name="effective_date"/>
+    <tableColumn id="8" name="market_cutoff_metadata"/>
+    <tableColumn id="9" name="units"/>
+    <tableColumn id="10" name="source_ids"/>
+    <tableColumn id="11" name="assumption_ids"/>
+    <tableColumn id="12" name="upstream_run_ids"/>
+    <tableColumn id="13" name="code_version"/>
+    <tableColumn id="14" name="input_hash"/>
+    <tableColumn id="15" name="confidence"/>
+    <tableColumn id="16" name="validation_status"/>
+    <tableColumn id="17" name="record_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -512,32 +474,32 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T_Data_Gaps" displayName="T_Data_Gaps" ref="A1:R2" headerRowCount="1">
   <autoFilter ref="A1:R2"/>
   <tableColumns count="18">
-    <tableColumn id="1" name="assumption_ids"/>
-    <tableColumn id="2" name="code_version"/>
-    <tableColumn id="3" name="confidence"/>
-    <tableColumn id="4" name="effective_date"/>
-    <tableColumn id="5" name="field"/>
-    <tableColumn id="6" name="input_hash"/>
-    <tableColumn id="7" name="market_cutoff_metadata"/>
-    <tableColumn id="8" name="next_action"/>
-    <tableColumn id="9" name="owner"/>
-    <tableColumn id="10" name="reason"/>
-    <tableColumn id="11" name="record_id"/>
-    <tableColumn id="12" name="run_id"/>
-    <tableColumn id="13" name="schema_version"/>
-    <tableColumn id="14" name="source_ids"/>
-    <tableColumn id="15" name="ticker"/>
-    <tableColumn id="16" name="units"/>
-    <tableColumn id="17" name="upstream_run_ids"/>
-    <tableColumn id="18" name="validation_status"/>
+    <tableColumn id="1" name="ticker"/>
+    <tableColumn id="2" name="field"/>
+    <tableColumn id="3" name="reason"/>
+    <tableColumn id="4" name="owner"/>
+    <tableColumn id="5" name="next_action"/>
+    <tableColumn id="6" name="schema_version"/>
+    <tableColumn id="7" name="run_id"/>
+    <tableColumn id="8" name="effective_date"/>
+    <tableColumn id="9" name="market_cutoff_metadata"/>
+    <tableColumn id="10" name="units"/>
+    <tableColumn id="11" name="source_ids"/>
+    <tableColumn id="12" name="assumption_ids"/>
+    <tableColumn id="13" name="upstream_run_ids"/>
+    <tableColumn id="14" name="code_version"/>
+    <tableColumn id="15" name="input_hash"/>
+    <tableColumn id="16" name="confidence"/>
+    <tableColumn id="17" name="validation_status"/>
+    <tableColumn id="18" name="record_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:I3" headerRowCount="1">
-  <autoFilter ref="A1:I3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:I4" headerRowCount="1">
+  <autoFilter ref="A1:I4"/>
   <tableColumns count="9">
     <tableColumn id="1" name="analysis_run_id"/>
     <tableColumn id="2" name="attempted_at"/>
@@ -896,7 +858,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NO_MATERIAL_CHANGE</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -920,7 +882,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20261012T105853333493Z-a85bcecf</t>
+          <t>20261026T152031546516Z-5f77f1ad</t>
         </is>
       </c>
     </row>
@@ -932,7 +894,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20261012T105838714078Z-1be18ab3</t>
+          <t>20261026T152031546516Z-5f77f1ad</t>
         </is>
       </c>
     </row>
@@ -944,26 +906,26 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BLOCKED_MODEL — Phase 2 not implemented</t>
+          <t>BLOCKED_MODEL — no research imported</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>assumption_ids</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
+          <t>15220.00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>ledger_cash</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -987,24 +949,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>code_version</t>
+          <t>equity_value</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>20450</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>total_assets</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SYNTHETIC</t>
+          <t>35670.00</t>
         </is>
       </c>
     </row>
@@ -1023,127 +985,127 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>data_gate_status</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+          <t>realized_gain</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>370.00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>effective_date</t>
+          <t>income_received</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>effective_positions</t>
+          <t>hhi</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2.817079537225711928057796264798504572169549182398410265909971202</t>
+          <t>0.3549775527405981551999330467895337784924767307703803779269612210</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>equity_value</t>
+          <t>effective_positions</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>20450</t>
+          <t>2.817079537225711928057796264798504572169549182398410265909971202</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>hhi</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>0.3549775527405981551999330467895337784924767307703803779269612210</t>
+          <t>sizing_status</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>holdings_timestamp</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-10-09T18:00:00+05:00</t>
+          <t>data_gate_status</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>income_received</t>
+          <t>sizing_reason</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>Executable sizing and integrated risk review require Phase 3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>input_hash</t>
+          <t>reconciliation_state</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+          <t>RECONCILED</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ledger_cash</t>
+          <t>mode</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>15220.00</t>
+          <t>DEMO</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>market_cutoff</t>
+          <t>holdings_timestamp</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-09T18:00:00+05:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>market_cutoff_metadata</t>
+          <t>market_cutoff</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1155,168 +1117,168 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>return_window_start</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DEMO</t>
+          <t>2026-10-08T18:00:00+05:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>return_window_end</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>2026-10-09T18:00:00+05:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>realized_gain</t>
+          <t>schema_version</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>370.00</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>reconciliation_state</t>
+          <t>run_id</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RECONCILED</t>
+          <t>20261026T152031546516Z-5f77f1ad</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>return_window_end</t>
+          <t>owner</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-09T18:00:00+05:00</t>
+          <t>portfolio</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>return_window_start</t>
+          <t>effective_date</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-08T18:00:00+05:00</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>run_id</t>
+          <t>market_cutoff_metadata</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>20261012T105838714078Z-1be18ab3</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>schema_version</t>
+          <t>units</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>PKR / shares / fraction as named</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>sizing_reason</t>
+          <t>source_ids</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Phase 1 does not implement executable sizing or risk review</t>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>sizing_status</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+          <t>assumption_ids</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>source_ids</t>
+          <t>upstream_run_ids</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>total_assets</t>
+          <t>code_version</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>35670.00</t>
+          <t>0.2.0</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>input_hash</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PKR / shares / fraction as named</t>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>upstream_run_ids</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>SYNTHETIC</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2061,6 +2023,51 @@
         </is>
       </c>
       <c r="I3" t="inlineStr">
+        <is>
+          <t>AI telemetry unknown; total wall time recorded externally after commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.04806</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>AI telemetry unknown; total wall time recorded externally after commit</t>
         </is>
@@ -2301,7 +2308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2320,23 +2327,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -2346,7 +2339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2365,23 +2358,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -2391,7 +2370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2410,23 +2389,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -2436,7 +2401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2455,23 +2420,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -2481,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2500,23 +2451,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -4204,6 +4141,51 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NOT_IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>No accepted model or live data migrated; see docs/migration.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4597,457 +4579,457 @@
   <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>effective_date</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>market_cutoff_metadata</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>source_ids</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>assumption_ids</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>upstream_run_ids</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>code_version</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>input_hash</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>effective_date</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>input_hash</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>market_cutoff_metadata</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>outcome</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>record_id</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>run_id</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>schema_version</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>source_ids</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>units</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>upstream_run_ids</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>validation_status</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>DEMO-BANK</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BLOCKED_MODEL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>valuation</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>No accepted Phase 2 model and verified inputs supplied</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PKR / shares / fraction as named</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>BLOCKED_MODEL</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>valuation</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Phase 2 adapter and verified inputs not supplied</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>coverage.0</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>20261012T105838714078Z-1be18ab3</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>DEMO-BANK</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>PKR / shares / fraction as named</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>VALIDATED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>DEMO-ENERGY</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BLOCKED_MODEL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>valuation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>No accepted Phase 2 model and verified inputs supplied</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PKR / shares / fraction as named</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>BLOCKED_MODEL</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>valuation</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Phase 2 adapter and verified inputs not supplied</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>coverage.1</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>20261012T105838714078Z-1be18ab3</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>DEMO-ENERGY</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>PKR / shares / fraction as named</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>VALIDATED</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>DEMO-INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BLOCKED_MODEL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>valuation</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>No accepted Phase 2 model and verified inputs supplied</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>PKR / shares / fraction as named</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>BLOCKED_MODEL</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>valuation</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Phase 2 adapter and verified inputs not supplied</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>coverage.2</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>20261012T105838714078Z-1be18ab3</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>DEMO-INDUSTRIAL</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>PKR / shares / fraction as named</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>VALIDATED</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>DEMO-LOSS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BLOCKED_MODEL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>valuation</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>No accepted Phase 2 model and verified inputs supplied</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>PKR / shares / fraction as named</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>BLOCKED_MODEL</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>valuation</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Phase 2 adapter and verified inputs not supplied</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>coverage.3</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>20261012T105838714078Z-1be18ab3</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>DEMO-LOSS</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>PKR / shares / fraction as named</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>VALIDATED</t>
         </is>
       </c>
     </row>
@@ -5068,207 +5050,207 @@
   <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>next_action</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>effective_date</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>market_cutoff_metadata</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>source_ids</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>assumption_ids</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>upstream_run_ids</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>code_version</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>input_hash</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>effective_date</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>field</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>input_hash</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>market_cutoff_metadata</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>next_action</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>record_id</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>run_id</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>schema_version</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>source_ids</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>units</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>upstream_run_ids</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>validation_status</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>risk_limits</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UNCONFIGURED_RISK_LIMITS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Confirm portfolio limits before sizing</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>PKR / shares / fraction as named</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>risk_limits</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Confirm portfolio limits before sizing</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>validation</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>UNCONFIGURED_RISK_LIMITS</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>data_gaps.0</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>20261012T105838714078Z-1be18ab3</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>PKR / shares / fraction as named</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>VALIDATED</t>
         </is>
       </c>
     </row>
@@ -5317,7 +5299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5472,6 +5454,53 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:20:31.594301+00:00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>LOCAL_ONLY</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>export-excel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
research: portfolio 20261026T152159474843Z-b2428599 [NO_MATERIAL_CHANGE]
Imported from local commit: f3cdbd7336ae9a2153b38a92e35b9e5d7f566de9
Original author: Investment Workspace <workspace@localhost> (2026-10-26T15:21:59Z)
File tree preserved exactly from the uploaded Git bundle.
</commit_message>
<xml_diff>
--- a/workbooks/Investment_Workspace.xlsx
+++ b/workbooks/Investment_Workspace.xlsx
@@ -194,8 +194,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:I4" headerRowCount="1">
-  <autoFilter ref="A1:I4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:I5" headerRowCount="1">
+  <autoFilter ref="A1:I5"/>
   <tableColumns count="9">
     <tableColumn id="1" name="cached_input_tokens"/>
     <tableColumn id="2" name="calculation_runtime_seconds"/>
@@ -448,23 +448,23 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T_Coverage" displayName="T_Coverage" ref="A1:Q5" headerRowCount="1">
   <autoFilter ref="A1:Q5"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="ticker"/>
-    <tableColumn id="2" name="outcome"/>
-    <tableColumn id="3" name="owner"/>
-    <tableColumn id="4" name="reason"/>
-    <tableColumn id="5" name="schema_version"/>
-    <tableColumn id="6" name="run_id"/>
-    <tableColumn id="7" name="effective_date"/>
-    <tableColumn id="8" name="market_cutoff_metadata"/>
-    <tableColumn id="9" name="units"/>
-    <tableColumn id="10" name="source_ids"/>
-    <tableColumn id="11" name="assumption_ids"/>
-    <tableColumn id="12" name="upstream_run_ids"/>
-    <tableColumn id="13" name="code_version"/>
-    <tableColumn id="14" name="input_hash"/>
-    <tableColumn id="15" name="confidence"/>
-    <tableColumn id="16" name="validation_status"/>
-    <tableColumn id="17" name="record_id"/>
+    <tableColumn id="1" name="assumption_ids"/>
+    <tableColumn id="2" name="code_version"/>
+    <tableColumn id="3" name="confidence"/>
+    <tableColumn id="4" name="effective_date"/>
+    <tableColumn id="5" name="input_hash"/>
+    <tableColumn id="6" name="market_cutoff_metadata"/>
+    <tableColumn id="7" name="outcome"/>
+    <tableColumn id="8" name="owner"/>
+    <tableColumn id="9" name="reason"/>
+    <tableColumn id="10" name="record_id"/>
+    <tableColumn id="11" name="run_id"/>
+    <tableColumn id="12" name="schema_version"/>
+    <tableColumn id="13" name="source_ids"/>
+    <tableColumn id="14" name="ticker"/>
+    <tableColumn id="15" name="units"/>
+    <tableColumn id="16" name="upstream_run_ids"/>
+    <tableColumn id="17" name="validation_status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -474,32 +474,32 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T_Data_Gaps" displayName="T_Data_Gaps" ref="A1:R2" headerRowCount="1">
   <autoFilter ref="A1:R2"/>
   <tableColumns count="18">
-    <tableColumn id="1" name="ticker"/>
-    <tableColumn id="2" name="field"/>
-    <tableColumn id="3" name="reason"/>
-    <tableColumn id="4" name="owner"/>
-    <tableColumn id="5" name="next_action"/>
-    <tableColumn id="6" name="schema_version"/>
-    <tableColumn id="7" name="run_id"/>
-    <tableColumn id="8" name="effective_date"/>
-    <tableColumn id="9" name="market_cutoff_metadata"/>
-    <tableColumn id="10" name="units"/>
-    <tableColumn id="11" name="source_ids"/>
-    <tableColumn id="12" name="assumption_ids"/>
-    <tableColumn id="13" name="upstream_run_ids"/>
-    <tableColumn id="14" name="code_version"/>
-    <tableColumn id="15" name="input_hash"/>
-    <tableColumn id="16" name="confidence"/>
-    <tableColumn id="17" name="validation_status"/>
-    <tableColumn id="18" name="record_id"/>
+    <tableColumn id="1" name="assumption_ids"/>
+    <tableColumn id="2" name="code_version"/>
+    <tableColumn id="3" name="confidence"/>
+    <tableColumn id="4" name="effective_date"/>
+    <tableColumn id="5" name="field"/>
+    <tableColumn id="6" name="input_hash"/>
+    <tableColumn id="7" name="market_cutoff_metadata"/>
+    <tableColumn id="8" name="next_action"/>
+    <tableColumn id="9" name="owner"/>
+    <tableColumn id="10" name="reason"/>
+    <tableColumn id="11" name="record_id"/>
+    <tableColumn id="12" name="run_id"/>
+    <tableColumn id="13" name="schema_version"/>
+    <tableColumn id="14" name="source_ids"/>
+    <tableColumn id="15" name="ticker"/>
+    <tableColumn id="16" name="units"/>
+    <tableColumn id="17" name="upstream_run_ids"/>
+    <tableColumn id="18" name="validation_status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:I4" headerRowCount="1">
-  <autoFilter ref="A1:I4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:I5" headerRowCount="1">
+  <autoFilter ref="A1:I5"/>
   <tableColumns count="9">
     <tableColumn id="1" name="analysis_run_id"/>
     <tableColumn id="2" name="attempted_at"/>
@@ -858,7 +858,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>NO_MATERIAL_CHANGE</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20261026T152031546516Z-5f77f1ad</t>
+          <t>20261026T152159474843Z-b2428599</t>
         </is>
       </c>
     </row>
@@ -913,19 +913,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>assumption_ids</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15220.00</t>
+          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ledger_cash</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -949,24 +949,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>equity_value</t>
+          <t>code_version</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>20450</t>
+          <t>0.2.0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>total_assets</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>35670.00</t>
+          <t>SYNTHETIC</t>
         </is>
       </c>
     </row>
@@ -985,127 +985,127 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>realized_gain</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>370.00</t>
+          <t>data_gate_status</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>income_received</t>
+          <t>effective_date</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hhi</t>
+          <t>effective_positions</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0.3549775527405981551999330467895337784924767307703803779269612210</t>
+          <t>2.817079537225711928057796264798504572169549182398410265909971202</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>effective_positions</t>
+          <t>equity_value</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2.817079537225711928057796264798504572169549182398410265909971202</t>
+          <t>20450</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sizing_status</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+          <t>hhi</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0.3549775527405981551999330467895337784924767307703803779269612210</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>data_gate_status</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+          <t>holdings_timestamp</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-09T18:00:00+05:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>sizing_reason</t>
+          <t>income_received</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Executable sizing and integrated risk review require Phase 3</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>reconciliation_state</t>
+          <t>input_hash</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RECONCILED</t>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>ledger_cash</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DEMO</t>
+          <t>15220.00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>holdings_timestamp</t>
+          <t>market_cutoff</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-09T18:00:00+05:00</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>market_cutoff</t>
+          <t>market_cutoff_metadata</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1117,168 +1117,168 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>return_window_start</t>
+          <t>mode</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-08T18:00:00+05:00</t>
+          <t>DEMO</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>return_window_end</t>
+          <t>owner</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-09T18:00:00+05:00</t>
+          <t>portfolio</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>schema_version</t>
+          <t>realized_gain</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>370.00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>run_id</t>
+          <t>reconciliation_state</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>20261026T152031546516Z-5f77f1ad</t>
+          <t>RECONCILED</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>return_window_end</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>2026-10-09T18:00:00+05:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>effective_date</t>
+          <t>return_window_start</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-08T18:00:00+05:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>market_cutoff_metadata</t>
+          <t>run_id</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>20261026T152031546516Z-5f77f1ad</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>schema_version</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PKR / shares / fraction as named</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>source_ids</t>
+          <t>sizing_reason</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+          <t>Executable sizing and integrated risk review require Phase 3</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>assumption_ids</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
+          <t>sizing_status</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>upstream_run_ids</t>
+          <t>source_ids</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>code_version</t>
+          <t>total_assets</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>35670.00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>input_hash</t>
+          <t>units</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+          <t>PKR / shares / fraction as named</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>upstream_run_ids</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SYNTHETIC</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2068,6 +2068,51 @@
         </is>
       </c>
       <c r="I4" t="inlineStr">
+        <is>
+          <t>AI telemetry unknown; total wall time recorded externally after commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.073542</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>20261026T152159474843Z-b2428599</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>AI telemetry unknown; total wall time recorded externally after commit</t>
         </is>
@@ -4579,457 +4624,457 @@
   <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>assumption_ids</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>code_version</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>effective_date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>input_hash</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>market_cutoff_metadata</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>source_ids</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>outcome</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>schema_version</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>run_id</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>effective_date</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>market_cutoff_metadata</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>units</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>source_ids</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>assumption_ids</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>upstream_run_ids</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>code_version</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>input_hash</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>confidence</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>validation_status</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>record_id</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>BLOCKED_MODEL</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>valuation</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>No accepted Phase 2 model and verified inputs supplied</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>coverage.0</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>DEMO-BANK</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>BLOCKED_MODEL</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>valuation</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>No accepted Phase 2 model and verified inputs supplied</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>20261026T152031546516Z-5f77f1ad</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>PKR / shares / fraction as named</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>0.2.0</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>VALIDATED</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>coverage.0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>BLOCKED_MODEL</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>valuation</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>No accepted Phase 2 model and verified inputs supplied</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>coverage.1</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>DEMO-ENERGY</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>BLOCKED_MODEL</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>valuation</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>No accepted Phase 2 model and verified inputs supplied</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>20261026T152031546516Z-5f77f1ad</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>PKR / shares / fraction as named</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>0.2.0</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>VALIDATED</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>coverage.1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>BLOCKED_MODEL</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>valuation</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No accepted Phase 2 model and verified inputs supplied</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>coverage.2</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>DEMO-INDUSTRIAL</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>BLOCKED_MODEL</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>valuation</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>No accepted Phase 2 model and verified inputs supplied</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>20261026T152031546516Z-5f77f1ad</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>PKR / shares / fraction as named</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>0.2.0</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>VALIDATED</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>coverage.2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>BLOCKED_MODEL</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>valuation</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No accepted Phase 2 model and verified inputs supplied</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>coverage.3</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
           <t>DEMO-LOSS</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>BLOCKED_MODEL</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>valuation</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>No accepted Phase 2 model and verified inputs supplied</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>20261026T152031546516Z-5f77f1ad</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>PKR / shares / fraction as named</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>0.2.0</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>VALIDATED</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>coverage.3</t>
         </is>
       </c>
     </row>
@@ -5050,207 +5095,207 @@
   <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>assumption_ids</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>code_version</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>effective_date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>input_hash</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>market_cutoff_metadata</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>next_action</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>source_ids</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>field</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>next_action</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>schema_version</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>run_id</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>effective_date</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>market_cutoff_metadata</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>units</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>source_ids</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>assumption_ids</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>upstream_run_ids</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>code_version</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>input_hash</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>confidence</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>validation_status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>record_id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>risk_limits</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Confirm portfolio limits before sizing</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UNCONFIGURED_RISK_LIMITS</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>data_gaps.0</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>risk_limits</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>UNCONFIGURED_RISK_LIMITS</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>validation</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Confirm portfolio limits before sizing</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>20261026T152031546516Z-5f77f1ad</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>PKR / shares / fraction as named</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0.2.0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>VALIDATED</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>data_gaps.0</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5501,6 +5546,53 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:21:59.548338+00:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>LOCAL_ONLY</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>20261026T152159474843Z-b2428599</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NO_MATERIAL_CHANGE</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>export-excel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
research: portfolio 20261026T155444530652Z-42e3cb45 [NO_MATERIAL_CHANGE]
Imported from local commit: dd49df2ec63729c8c238567bcf048c6531a41762
Original author: Investment Workspace <workspace@localhost> (2026-10-26T15:54:46Z)
File tree preserved exactly from the uploaded Git bundle.
</commit_message>
<xml_diff>
--- a/workbooks/Investment_Workspace.xlsx
+++ b/workbooks/Investment_Workspace.xlsx
@@ -26,17 +26,24 @@
     <sheet name="Entry_Levels" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="Dividend_Calendar" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Top_10" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Watchlist" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Catalysts" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="RS_Trend" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Sector_Rotation" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Mean_Reversion" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Macro" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Scenarios" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Portfolio_Risk" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="IC_Actions" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Retirement" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Cross_Asset" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="RS_Trend" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Sector_Rotation" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Mean_Reversion" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Macro" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Scenarios" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="News_Impact" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Portfolio_Risk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Correlations" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Watchlist" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Catalysts" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="IC_Actions" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Refresh_Queue" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="Event_Propagation" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="Backtests" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="Backtest_Trades" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="Alerts" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="Retirement" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="Cross_Asset" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reconciliation'!$A$1:$B$1</definedName>
@@ -47,6 +54,22 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Entry_Levels'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Dividend_Calendar'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Top_10'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'RS_Trend'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Sector_Rotation'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Mean_Reversion'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Macro'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Scenarios'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'News_Impact'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'Portfolio_Risk'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'Correlations'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'Watchlist'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Catalysts'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'IC_Actions'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'Refresh_Queue'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'Event_Propagation'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="32" hidden="1">'Backtests'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'Backtest_Trades'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="34" hidden="1">'Alerts'!$A$1:$B$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -183,8 +206,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Dashboard" displayName="T_Dashboard" ref="A1:B39" headerRowCount="1">
-  <autoFilter ref="A1:B39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Dashboard" displayName="T_Dashboard" ref="A1:B40" headerRowCount="1">
+  <autoFilter ref="A1:B40"/>
   <tableColumns count="2">
     <tableColumn id="1" name="metric"/>
     <tableColumn id="2" name="value"/>
@@ -194,8 +217,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:I5" headerRowCount="1">
-  <autoFilter ref="A1:I5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:I6" headerRowCount="1">
+  <autoFilter ref="A1:I6"/>
   <tableColumns count="9">
     <tableColumn id="1" name="cached_input_tokens"/>
     <tableColumn id="2" name="calculation_runtime_seconds"/>
@@ -229,7 +252,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T_Watchlist" displayName="T_Watchlist" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T_Retirement" displayName="T_Retirement" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -240,73 +263,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T_Catalysts" displayName="T_Catalysts" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="T_RS_Trend" displayName="T_RS_Trend" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="T_Sector_Rotation" displayName="T_Sector_Rotation" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="T_Mean_Reversion" displayName="T_Mean_Reversion" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="T_Macro" displayName="T_Macro" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="T_Scenarios" displayName="T_Scenarios" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="T_Portfolio_Risk" displayName="T_Portfolio_Risk" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T_Cross_Asset" displayName="T_Cross_Asset" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="status"/>
@@ -337,39 +294,6 @@
     <tableColumn id="15" name="run_id"/>
     <tableColumn id="16" name="effective_date"/>
     <tableColumn id="17" name="source_ids"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="T_IC_Actions" displayName="T_IC_Actions" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="T_Retirement" displayName="T_Retirement" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="T_Cross_Asset" displayName="T_Cross_Asset" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -498,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:I5" headerRowCount="1">
-  <autoFilter ref="A1:I5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:I6" headerRowCount="1">
+  <autoFilter ref="A1:I6"/>
   <tableColumns count="9">
     <tableColumn id="1" name="analysis_run_id"/>
     <tableColumn id="2" name="attempted_at"/>
@@ -819,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -882,7 +806,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20261026T152159474843Z-b2428599</t>
+          <t>20261026T155444530652Z-42e3cb45</t>
         </is>
       </c>
     </row>
@@ -1291,6 +1215,18 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>VALIDATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>integration_status</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>BLOCKED_INPUT — no integration imported</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2113,6 +2049,51 @@
         </is>
       </c>
       <c r="I5" t="inlineStr">
+        <is>
+          <t>AI telemetry unknown; total wall time recorded externally after commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.059103</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>20261026T155444530652Z-42e3cb45</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>AI telemetry unknown; total wall time recorded externally after commit</t>
         </is>
@@ -2915,7 +2896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2934,23 +2915,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -2960,7 +2927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2979,23 +2946,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -3005,7 +2958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3024,23 +2977,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -3050,7 +2989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3069,23 +3008,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -3095,7 +3020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3114,23 +3039,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -3140,7 +3051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3159,23 +3070,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -3185,7 +3082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3204,23 +3101,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -3230,7 +3113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3249,23 +3132,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -3275,7 +3144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3294,23 +3163,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -3320,7 +3175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3339,23 +3194,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -4192,6 +4033,237 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NOT_IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>No accepted model or live data migrated; see docs/migration.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5344,7 +5416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5593,6 +5665,53 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>20261026T152031546516Z-5f77f1ad</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:54:44.589699+00:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>LOCAL_ONLY</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>20261026T155444530652Z-42e3cb45</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>NO_MATERIAL_CHANGE</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>export-excel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
research: portfolio 20261026T225805178235Z-8f6aa76b [SUCCESS]
Imported from local commit: 036779df90a0168190e77501a4e75c4999470811
Original author: Investment Workspace <workspace@localhost> (2026-10-26T22:58:05Z)
File tree preserved exactly from the uploaded Git bundle.
</commit_message>
<xml_diff>
--- a/workbooks/Investment_Workspace.xlsx
+++ b/workbooks/Investment_Workspace.xlsx
@@ -26,24 +26,32 @@
     <sheet name="Entry_Levels" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="Dividend_Calendar" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Top_10" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="RS_Trend" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Sector_Rotation" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Mean_Reversion" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Macro" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Scenarios" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="News_Impact" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Portfolio_Risk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Correlations" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Watchlist" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Catalysts" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="IC_Actions" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="Refresh_Queue" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="Event_Propagation" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="Backtests" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="Backtest_Trades" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="Alerts" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="Retirement" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="Cross_Asset" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="Forward_Bridge" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="RS_Trend" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Sector_Rotation" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Mean_Reversion" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Macro" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Scenarios" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="News_Impact" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Portfolio_Risk" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Correlations" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Watchlist" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Catalysts" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="IC_Actions" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="Refresh_Queue" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="Event_Propagation" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="Backtests" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="Backtest_Trades" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="Alerts" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="Wealth_Assets" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="Wealth_Flows" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="Retirement" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="Retirement_Summary" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="Cross_Asset" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="Asset_Correlations" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="Financial_Facts" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Evidence_Library" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="Readiness" sheetId="45" state="visible" r:id="rId45"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reconciliation'!$A$1:$B$1</definedName>
@@ -54,22 +62,31 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Entry_Levels'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Dividend_Calendar'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Top_10'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'RS_Trend'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Sector_Rotation'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Mean_Reversion'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Macro'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Scenarios'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'News_Impact'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'Portfolio_Risk'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'Correlations'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'Watchlist'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Catalysts'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'IC_Actions'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'Refresh_Queue'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'Event_Propagation'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="32" hidden="1">'Backtests'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'Backtest_Trades'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="34" hidden="1">'Alerts'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Forward_Bridge'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'RS_Trend'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Sector_Rotation'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Mean_Reversion'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Macro'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'Scenarios'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'News_Impact'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'Portfolio_Risk'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'Correlations'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Watchlist'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'Catalysts'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'IC_Actions'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'Refresh_Queue'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="32" hidden="1">'Event_Propagation'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'Backtests'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="34" hidden="1">'Backtest_Trades'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="35" hidden="1">'Alerts'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="36" hidden="1">'Wealth_Assets'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="37" hidden="1">'Wealth_Flows'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="38" hidden="1">'Retirement'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="39" hidden="1">'Retirement_Summary'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="40" hidden="1">'Cross_Asset'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="41" hidden="1">'Asset_Correlations'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="42" hidden="1">'Financial_Facts'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="43" hidden="1">'Evidence_Library'!$A$1:$B$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -217,9 +234,9 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:I6" headerRowCount="1">
-  <autoFilter ref="A1:I6"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:N7" headerRowCount="1">
+  <autoFilter ref="A1:N7"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="cached_input_tokens"/>
     <tableColumn id="2" name="calculation_runtime_seconds"/>
     <tableColumn id="3" name="cost"/>
@@ -229,6 +246,11 @@
     <tableColumn id="7" name="run_id"/>
     <tableColumn id="8" name="runtime_seconds"/>
     <tableColumn id="9" name="telemetry"/>
+    <tableColumn id="10" name="phase_runtime_seconds"/>
+    <tableColumn id="11" name="calculation_units"/>
+    <tableColumn id="12" name="cache_hits"/>
+    <tableColumn id="13" name="cache_arithmetic_verified"/>
+    <tableColumn id="14" name="deferred_units"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -252,22 +274,11 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T_Retirement" displayName="T_Retirement" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T_Readiness" displayName="T_Readiness" ref="A1:B9" headerRowCount="1">
+  <autoFilter ref="A1:B9"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T_Cross_Asset" displayName="T_Cross_Asset" ref="A1:B2" headerRowCount="1">
-  <autoFilter ref="A1:B2"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="status"/>
-    <tableColumn id="2" name="reason"/>
+    <tableColumn id="1" name="dimension"/>
+    <tableColumn id="2" name="value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -398,33 +409,33 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T_Data_Gaps" displayName="T_Data_Gaps" ref="A1:R2" headerRowCount="1">
   <autoFilter ref="A1:R2"/>
   <tableColumns count="18">
-    <tableColumn id="1" name="assumption_ids"/>
-    <tableColumn id="2" name="code_version"/>
-    <tableColumn id="3" name="confidence"/>
-    <tableColumn id="4" name="effective_date"/>
-    <tableColumn id="5" name="field"/>
-    <tableColumn id="6" name="input_hash"/>
-    <tableColumn id="7" name="market_cutoff_metadata"/>
-    <tableColumn id="8" name="next_action"/>
-    <tableColumn id="9" name="owner"/>
-    <tableColumn id="10" name="reason"/>
-    <tableColumn id="11" name="record_id"/>
-    <tableColumn id="12" name="run_id"/>
-    <tableColumn id="13" name="schema_version"/>
-    <tableColumn id="14" name="source_ids"/>
-    <tableColumn id="15" name="ticker"/>
-    <tableColumn id="16" name="units"/>
-    <tableColumn id="17" name="upstream_run_ids"/>
-    <tableColumn id="18" name="validation_status"/>
+    <tableColumn id="1" name="ticker"/>
+    <tableColumn id="2" name="field"/>
+    <tableColumn id="3" name="reason"/>
+    <tableColumn id="4" name="owner"/>
+    <tableColumn id="5" name="next_action"/>
+    <tableColumn id="6" name="schema_version"/>
+    <tableColumn id="7" name="run_id"/>
+    <tableColumn id="8" name="effective_date"/>
+    <tableColumn id="9" name="market_cutoff_metadata"/>
+    <tableColumn id="10" name="units"/>
+    <tableColumn id="11" name="source_ids"/>
+    <tableColumn id="12" name="assumption_ids"/>
+    <tableColumn id="13" name="upstream_run_ids"/>
+    <tableColumn id="14" name="code_version"/>
+    <tableColumn id="15" name="input_hash"/>
+    <tableColumn id="16" name="confidence"/>
+    <tableColumn id="17" name="validation_status"/>
+    <tableColumn id="18" name="record_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:I6" headerRowCount="1">
-  <autoFilter ref="A1:I6"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:J7" headerRowCount="1">
+  <autoFilter ref="A1:J7"/>
+  <tableColumns count="10">
     <tableColumn id="1" name="analysis_run_id"/>
     <tableColumn id="2" name="attempted_at"/>
     <tableColumn id="3" name="error"/>
@@ -434,21 +445,23 @@
     <tableColumn id="7" name="run_id"/>
     <tableColumn id="8" name="status"/>
     <tableColumn id="9" name="workflow"/>
+    <tableColumn id="10" name="dataset_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="T_Change_Log" displayName="T_Change_Log" ref="A1:F17" headerRowCount="1">
-  <autoFilter ref="A1:F17"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="T_Change_Log" displayName="T_Change_Log" ref="A1:G18" headerRowCount="1">
+  <autoFilter ref="A1:G18"/>
+  <tableColumns count="7">
     <tableColumn id="1" name="field"/>
     <tableColumn id="2" name="new"/>
     <tableColumn id="3" name="previous"/>
     <tableColumn id="4" name="run_id"/>
     <tableColumn id="5" name="source_ids"/>
     <tableColumn id="6" name="ticker"/>
+    <tableColumn id="7" name="change_type"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -782,7 +795,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NO_MATERIAL_CHANGE</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -806,7 +819,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20261026T155444530652Z-42e3cb45</t>
+          <t>20261026T225805178235Z-8f6aa76b</t>
         </is>
       </c>
     </row>
@@ -818,7 +831,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20261026T152031546516Z-5f77f1ad</t>
+          <t>20261026T225805178235Z-8f6aa76b</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1253,6 +1266,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1286,6 +1300,11 @@
           <t>ticker</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>change_type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1318,6 +1337,11 @@
           <t>DEMO-BANK</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1350,6 +1374,11 @@
           <t>DEMO-BANK</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1382,6 +1411,11 @@
           <t>DEMO-BANK</t>
         </is>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1414,6 +1448,11 @@
           <t>DEMO-BANK</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1446,6 +1485,11 @@
           <t>DEMO-ENERGY</t>
         </is>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1478,6 +1522,11 @@
           <t>DEMO-ENERGY</t>
         </is>
       </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1510,6 +1559,11 @@
           <t>DEMO-ENERGY</t>
         </is>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1542,6 +1596,11 @@
           <t>DEMO-ENERGY</t>
         </is>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1574,6 +1633,11 @@
           <t>DEMO-INDUSTRIAL</t>
         </is>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1606,6 +1670,11 @@
           <t>DEMO-INDUSTRIAL</t>
         </is>
       </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1638,6 +1707,11 @@
           <t>DEMO-INDUSTRIAL</t>
         </is>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1670,6 +1744,11 @@
           <t>DEMO-INDUSTRIAL</t>
         </is>
       </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1702,6 +1781,11 @@
           <t>DEMO-LOSS</t>
         </is>
       </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1734,6 +1818,11 @@
           <t>DEMO-LOSS</t>
         </is>
       </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1766,6 +1855,11 @@
           <t>DEMO-LOSS</t>
         </is>
       </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1796,6 +1890,48 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>DEMO-LOSS</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>evidence_registry</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>4bb4c6d66e21226e8175622ccd49599b6206624a0547584c5501232196516855</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>EVIDENCE</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1825,6 +1961,11 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1873,6 +2014,31 @@
           <t>telemetry</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>phase_runtime_seconds</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>calculation_units</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>cache_hits</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>cache_arithmetic_verified</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>deferred_units</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1918,6 +2084,31 @@
           <t>AI telemetry unknown; total wall time recorded externally after commit</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1963,6 +2154,31 @@
           <t>AI telemetry unknown; total wall time recorded externally after commit</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2008,6 +2224,31 @@
           <t>AI telemetry unknown; total wall time recorded externally after commit</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2053,6 +2294,31 @@
           <t>AI telemetry unknown; total wall time recorded externally after commit</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2097,6 +2363,93 @@
         <is>
           <t>AI telemetry unknown; total wall time recorded externally after commit</t>
         </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.045383</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>AI telemetry unknown; total wall time recorded externally after commit</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>{"integration": 5e-06, "portfolio": 0.000254, "valuation": 6e-06, "wealth": 1e-06}</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4219,7 +4572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4238,23 +4591,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -4264,7 +4603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4283,23 +4622,71 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOT_IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No accepted model or live data migrated; see docs/migration.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -4367,6 +4754,288 @@
       </c>
       <c r="E2" s="3" t="n">
         <v>370</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>calculation_status</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>compatibility</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NOT_MIGRATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>coverage</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"cross-asset": "BLOCKED_INPUT", "ic": "BLOCKED_INPUT", "macro": "BLOCKED_INPUT", "portfolio": "PARTIAL", "retirement": "BLOCKED_INPUT", "timing": "BLOCKED_INPUT", "valuation": "BLOCKED_INPUT", "watchlist": "BLOCKED_INPUT"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>{"dataset_id": "legacy.demo", "mode": "DEMO"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>dependencies</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>[{"next_action": "Confirm portfolio limits before sizing", "owner": "validation", "reason": "UNCONFIGURED_RISK_LIMITS", "ticker": null}, {"next_action": "Supply and reconcile the real legacy datastore", "owner": "migration", "reason": "LEGACY_PARITY_REQUIRED"}, {"next_action": "Import the original PRD source document with hash and locator", "owner": "evidence", "reason": "MISSING_EVIDENCE_CONTRACT"}, {"next_action": "Import the original PRD source document with hash and locator", "owner": "evidence", "reason": "MISSING_REPLACEMENT_PROMPTS"}, {"next_action": "Import the original PRD source document with hash and locator", "owner": "evidence", "reason": "MISSING_VALUATION_RERUN"}, {"next_action": "Import publication/access metadata, ownership, coverage dates and source URL or original hash", "owner": "evidence", "reason": "INCOMPLETE_PROVENANCE"}, {"next_action": "Confirm production dataset, manual parity, source coverage and publication policy", "owner": "deployment", "reason": "NOT_ACTIVATED"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>deployment</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>evaluation_as_of</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>schedules_enabled</t>
+        </is>
+      </c>
+      <c r="B9" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5167,207 +5836,207 @@
   <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>next_action</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>effective_date</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>market_cutoff_metadata</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>source_ids</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>assumption_ids</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>upstream_run_ids</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>code_version</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>input_hash</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>effective_date</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>field</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>input_hash</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>market_cutoff_metadata</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>next_action</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>record_id</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>run_id</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>schema_version</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>source_ids</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>units</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>upstream_run_ids</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>validation_status</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>risk_limits</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UNCONFIGURED_RISK_LIMITS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Confirm portfolio limits before sizing</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>PKR / shares / fraction as named</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>0.2.0</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0.4.0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>risk_limits</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Confirm portfolio limits before sizing</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>validation</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>UNCONFIGURED_RISK_LIMITS</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>data_gaps.0</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>20261026T152031546516Z-5f77f1ad</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>PKR / shares / fraction as named</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>VALIDATED</t>
         </is>
       </c>
     </row>
@@ -5416,7 +6085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5428,6 +6097,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5476,6 +6146,11 @@
           <t>workflow</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dataset_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5523,6 +6198,11 @@
           <t>init-demo</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5570,6 +6250,11 @@
           <t>portfolio</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5617,6 +6302,11 @@
           <t>export-excel</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5664,6 +6354,11 @@
           <t>export-excel</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5709,6 +6404,63 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>export-excel</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-26T22:58:05.223532+00:00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>LOCAL_ONLY</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>export-excel</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>legacy.demo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
research: portfolio 20261027T030318603078Z-fbb26a6c [NO_MATERIAL_CHANGE]
Imported from local commit: 35df12feb504813bb2156a0de9482dd5e2ddab86
Original author: Investment Workspace <workspace@localhost> (2026-10-27T03:03:19Z)
File tree preserved exactly from the uploaded Git bundle.
</commit_message>
<xml_diff>
--- a/workbooks/Investment_Workspace.xlsx
+++ b/workbooks/Investment_Workspace.xlsx
@@ -234,8 +234,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:N7" headerRowCount="1">
-  <autoFilter ref="A1:N7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:N8" headerRowCount="1">
+  <autoFilter ref="A1:N8"/>
   <tableColumns count="14">
     <tableColumn id="1" name="cached_input_tokens"/>
     <tableColumn id="2" name="calculation_runtime_seconds"/>
@@ -246,11 +246,11 @@
     <tableColumn id="7" name="run_id"/>
     <tableColumn id="8" name="runtime_seconds"/>
     <tableColumn id="9" name="telemetry"/>
-    <tableColumn id="10" name="phase_runtime_seconds"/>
-    <tableColumn id="11" name="calculation_units"/>
-    <tableColumn id="12" name="cache_hits"/>
-    <tableColumn id="13" name="cache_arithmetic_verified"/>
-    <tableColumn id="14" name="deferred_units"/>
+    <tableColumn id="10" name="cache_arithmetic_verified"/>
+    <tableColumn id="11" name="cache_hits"/>
+    <tableColumn id="12" name="calculation_units"/>
+    <tableColumn id="13" name="deferred_units"/>
+    <tableColumn id="14" name="phase_runtime_seconds"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -409,32 +409,32 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T_Data_Gaps" displayName="T_Data_Gaps" ref="A1:R2" headerRowCount="1">
   <autoFilter ref="A1:R2"/>
   <tableColumns count="18">
-    <tableColumn id="1" name="ticker"/>
-    <tableColumn id="2" name="field"/>
-    <tableColumn id="3" name="reason"/>
-    <tableColumn id="4" name="owner"/>
-    <tableColumn id="5" name="next_action"/>
-    <tableColumn id="6" name="schema_version"/>
-    <tableColumn id="7" name="run_id"/>
-    <tableColumn id="8" name="effective_date"/>
-    <tableColumn id="9" name="market_cutoff_metadata"/>
-    <tableColumn id="10" name="units"/>
-    <tableColumn id="11" name="source_ids"/>
-    <tableColumn id="12" name="assumption_ids"/>
-    <tableColumn id="13" name="upstream_run_ids"/>
-    <tableColumn id="14" name="code_version"/>
-    <tableColumn id="15" name="input_hash"/>
-    <tableColumn id="16" name="confidence"/>
-    <tableColumn id="17" name="validation_status"/>
-    <tableColumn id="18" name="record_id"/>
+    <tableColumn id="1" name="assumption_ids"/>
+    <tableColumn id="2" name="code_version"/>
+    <tableColumn id="3" name="confidence"/>
+    <tableColumn id="4" name="effective_date"/>
+    <tableColumn id="5" name="field"/>
+    <tableColumn id="6" name="input_hash"/>
+    <tableColumn id="7" name="market_cutoff_metadata"/>
+    <tableColumn id="8" name="next_action"/>
+    <tableColumn id="9" name="owner"/>
+    <tableColumn id="10" name="reason"/>
+    <tableColumn id="11" name="record_id"/>
+    <tableColumn id="12" name="run_id"/>
+    <tableColumn id="13" name="schema_version"/>
+    <tableColumn id="14" name="source_ids"/>
+    <tableColumn id="15" name="ticker"/>
+    <tableColumn id="16" name="units"/>
+    <tableColumn id="17" name="upstream_run_ids"/>
+    <tableColumn id="18" name="validation_status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:J7" headerRowCount="1">
-  <autoFilter ref="A1:J7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:J8" headerRowCount="1">
+  <autoFilter ref="A1:J8"/>
   <tableColumns count="10">
     <tableColumn id="1" name="analysis_run_id"/>
     <tableColumn id="2" name="attempted_at"/>
@@ -795,7 +795,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>NO_MATERIAL_CHANGE</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20261026T225805178235Z-8f6aa76b</t>
+          <t>20261027T030318603078Z-fbb26a6c</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1961,11 +1961,11 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2016,27 +2016,27 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>cache_arithmetic_verified</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>cache_hits</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>calculation_units</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>deferred_units</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>phase_runtime_seconds</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>calculation_units</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>cache_hits</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>cache_arithmetic_verified</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>deferred_units</t>
         </is>
       </c>
     </row>
@@ -2434,10 +2434,8 @@
           <t>AI telemetry unknown; total wall time recorded externally after commit</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>{"integration": 5e-06, "portfolio": 0.000254, "valuation": 6e-06, "wealth": 1e-06}</t>
-        </is>
+      <c r="J7" t="n">
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -2448,8 +2446,72 @@
       <c r="M7" t="n">
         <v>0</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>{"integration": 5e-06, "portfolio": 0.000254, "valuation": 6e-06, "wealth": 1e-06}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.09155199999999999</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>20261027T030318603078Z-fbb26a6c</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>AI telemetry unknown; total wall time recorded externally after commit</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
         <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>{"integration": 4e-06, "portfolio": 0.000297, "valuation": 1.1e-05, "wealth": 1e-06}</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -4952,7 +5014,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>NO_MATERIAL_CHANGE</t>
         </is>
       </c>
     </row>
@@ -5836,207 +5898,207 @@
   <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>assumption_ids</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>code_version</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>effective_date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>input_hash</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>market_cutoff_metadata</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>next_action</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>source_ids</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>field</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>next_action</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>schema_version</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>run_id</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>effective_date</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>market_cutoff_metadata</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>units</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>source_ids</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>assumption_ids</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>upstream_run_ids</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>code_version</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>input_hash</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>confidence</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>validation_status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>record_id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>0.4.0</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>risk_limits</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Confirm portfolio limits before sizing</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>UNCONFIGURED_RISK_LIMITS</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>validation</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Confirm portfolio limits before sizing</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>data_gaps.0</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>20261026T225805178235Z-8f6aa76b</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>PKR / shares / fraction as named</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>["demo.closing.v1", "demo.ledger.v1", "demo.opening.v1", "demo.prices.v1", "input.f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892"]</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>["policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b"]</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0.4.0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>VALIDATED</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>data_gaps.0</t>
         </is>
       </c>
     </row>
@@ -6085,7 +6147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6464,6 +6526,58 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-27T03:03:18.691867+00:00</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>LOCAL_ONLY</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>20261027T030318603078Z-fbb26a6c</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NO_MATERIAL_CHANGE</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>export-excel</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>legacy.demo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
research: portfolio 20261031T084234360869Z-775910bd [NO_MATERIAL_CHANGE]
Imported from local commit: 3286adf2a5f08d4e7b0878db39bb1319ef6a85a5
Exact file tree preserved. Production and R2 policies remain disabled.
</commit_message>
<xml_diff>
--- a/workbooks/Investment_Workspace.xlsx
+++ b/workbooks/Investment_Workspace.xlsx
@@ -94,8 +94,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00;[Red](#,##0.00)"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00;[Red](#,##0.00)"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -110,7 +112,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -127,6 +129,11 @@
         <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -140,12 +147,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -234,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:N8" headerRowCount="1">
-  <autoFilter ref="A1:N8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:N9" headerRowCount="1">
+  <autoFilter ref="A1:N9"/>
   <tableColumns count="14">
     <tableColumn id="1" name="cached_input_tokens"/>
     <tableColumn id="2" name="calculation_runtime_seconds"/>
@@ -433,8 +442,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:J8" headerRowCount="1">
-  <autoFilter ref="A1:J8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:J9" headerRowCount="1">
+  <autoFilter ref="A1:J9"/>
   <tableColumns count="10">
     <tableColumn id="1" name="analysis_run_id"/>
     <tableColumn id="2" name="attempted_at"/>
@@ -819,7 +828,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20261027T030318603078Z-fbb26a6c</t>
+          <t>20261031T084234360869Z-775910bd</t>
         </is>
       </c>
     </row>
@@ -841,7 +850,7 @@
           <t>valuation_status</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>BLOCKED_MODEL — no research imported</t>
         </is>
@@ -1237,7 +1246,7 @@
           <t>integration_status</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>BLOCKED_INPUT — no integration imported</t>
         </is>
@@ -1949,7 +1958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2511,6 +2520,68 @@
       <c r="N8" t="inlineStr">
         <is>
           <t>{"integration": 4e-06, "portfolio": 0.000297, "valuation": 1.1e-05, "wealth": 1e-06}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.0457</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>20261031T084234360869Z-775910bd</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>AI telemetry unknown; total wall time recorded externally after commit</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>{"integration": 4e-06, "portfolio": 0.00026, "valuation": 1e-05, "wealth": 2e-06}</t>
         </is>
       </c>
     </row>
@@ -2620,10 +2691,8 @@
           <t>policy.2df429d66e495fb1169bd0ae55c856a17ff340d040bfaf4c4b632837f763676b</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="B2" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -3038,10 +3107,8 @@
       <c r="F2" s="3" t="n">
         <v>125</v>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="G2" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>10000</v>
@@ -3049,13 +3116,13 @@
       <c r="I2" s="3" t="n">
         <v>2000</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J2" s="5" t="n">
         <v>0.25</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="K2" s="5" t="n">
         <v>0.4889975550122249</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="L2" s="5" t="n">
         <v>0.2803476310625175</v>
       </c>
       <c r="M2" t="inlineStr">
@@ -3073,10 +3140,8 @@
           <t>20261012T105838714078Z-1be18ab3</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="P2" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -3109,10 +3174,8 @@
       <c r="F3" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="G3" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>5500</v>
@@ -3120,13 +3183,13 @@
       <c r="I3" s="3" t="n">
         <v>450</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="5" t="n">
         <v>0.0891089108910891</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="K3" s="5" t="n">
         <v>0.2689486552567237</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="L3" s="5" t="n">
         <v>0.1541911970843846</v>
       </c>
       <c r="M3" t="inlineStr">
@@ -3144,10 +3207,8 @@
           <t>20261012T105838714078Z-1be18ab3</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="P3" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -3180,10 +3241,8 @@
       <c r="F4" s="3" t="n">
         <v>105</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="G4" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>4200</v>
@@ -3191,13 +3250,13 @@
       <c r="I4" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="5" t="n">
         <v>0.2053789731051345</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="5" t="n">
         <v>0.1177460050462574</v>
       </c>
       <c r="M4" t="inlineStr">
@@ -3215,10 +3274,8 @@
           <t>20261012T105838714078Z-1be18ab3</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="P4" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -3251,10 +3308,8 @@
       <c r="F5" s="3" t="n">
         <v>75</v>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="G5" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>750</v>
@@ -3262,13 +3317,13 @@
       <c r="I5" s="3" t="n">
         <v>-250</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="5" t="n">
         <v>-0.25</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K5" s="5" t="n">
         <v>0.03667481662591687</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="L5" s="5" t="n">
         <v>0.02102607232968881</v>
       </c>
       <c r="M5" t="inlineStr">
@@ -3286,10 +3341,8 @@
           <t>20261012T105838714078Z-1be18ab3</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="P5" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -3813,15 +3866,13 @@
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="F2" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>0</v>
@@ -3875,10 +3926,8 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="S2" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -3941,15 +3990,13 @@
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="F3" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>50</v>
@@ -4003,10 +4050,8 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="S3" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -4069,15 +4114,13 @@
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="F4" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>30</v>
@@ -4131,10 +4174,8 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="S4" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -4197,15 +4238,13 @@
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="F5" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>0</v>
@@ -4259,10 +4298,8 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="S5" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -4325,15 +4362,13 @@
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="F6" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -4385,10 +4420,8 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="S6" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -5186,10 +5219,8 @@
           <t>data/evidence/blobs/f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892.json</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
+      <c r="C2" s="4" t="n">
+        <v>46303</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5233,10 +5264,8 @@
           <t>data/evidence/blobs/f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892.json</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="C3" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5280,10 +5309,8 @@
           <t>data/evidence/blobs/f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892.json</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="C4" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5327,10 +5354,8 @@
           <t>data/evidence/blobs/f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892.json</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="C5" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5374,10 +5399,8 @@
           <t>data/evidence/blobs/f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892.json</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="C6" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5544,27 +5567,25 @@
           <t>0.2.0</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="4" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>BLOCKED_MODEL</t>
         </is>
@@ -5631,27 +5652,25 @@
           <t>0.2.0</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="4" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>BLOCKED_MODEL</t>
         </is>
@@ -5718,27 +5737,25 @@
           <t>0.2.0</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="4" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>BLOCKED_MODEL</t>
         </is>
@@ -5805,27 +5822,25 @@
           <t>0.2.0</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="4" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>BLOCKED_MODEL</t>
         </is>
@@ -6021,15 +6036,13 @@
           <t>0.4.0</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="D2" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -6147,7 +6160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6235,10 +6248,8 @@
           <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="E2" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6287,10 +6298,8 @@
           <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="E3" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6339,10 +6348,8 @@
           <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="E4" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -6391,10 +6398,8 @@
           <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="E5" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -6443,10 +6448,8 @@
           <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="E6" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -6495,10 +6498,8 @@
           <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="E7" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -6547,10 +6548,8 @@
           <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
+      <c r="E8" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -6573,6 +6572,56 @@
         </is>
       </c>
       <c r="J8" t="inlineStr">
+        <is>
+          <t>legacy.demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-31T08:42:34.406469+00:00</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>LOCAL_ONLY</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>20261031T084234360869Z-775910bd</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NO_MATERIAL_CHANGE</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>export-excel</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>legacy.demo</t>
         </is>

</xml_diff>

<commit_message>
research: portfolio 20261031T085618170933Z-fbe64605 [NO_MATERIAL_CHANGE]
Imported from local commit be49a000e05162076517afbbbeded6254838b3c6
</commit_message>
<xml_diff>
--- a/workbooks/Investment_Workspace.xlsx
+++ b/workbooks/Investment_Workspace.xlsx
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:N9" headerRowCount="1">
-  <autoFilter ref="A1:N9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:N10" headerRowCount="1">
+  <autoFilter ref="A1:N10"/>
   <tableColumns count="14">
     <tableColumn id="1" name="cached_input_tokens"/>
     <tableColumn id="2" name="calculation_runtime_seconds"/>
@@ -442,8 +442,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:J9" headerRowCount="1">
-  <autoFilter ref="A1:J9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:J10" headerRowCount="1">
+  <autoFilter ref="A1:J10"/>
   <tableColumns count="10">
     <tableColumn id="1" name="analysis_run_id"/>
     <tableColumn id="2" name="attempted_at"/>
@@ -828,7 +828,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20261031T084234360869Z-775910bd</t>
+          <t>20261031T085618170933Z-fbe64605</t>
         </is>
       </c>
     </row>
@@ -1958,7 +1958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2582,6 +2582,68 @@
       <c r="N9" t="inlineStr">
         <is>
           <t>{"integration": 4e-06, "portfolio": 0.00026, "valuation": 1e-05, "wealth": 2e-06}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.055081</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>20261031T085618170933Z-fbe64605</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>AI telemetry unknown; total wall time recorded externally after commit</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>{"integration": 4e-06, "portfolio": 0.000417, "valuation": 9e-06, "wealth": 2e-06}</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6627,6 +6689,56 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-31T08:56:18.225876+00:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>LOCAL_ONLY</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>20261031T085618170933Z-fbe64605</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>NO_MATERIAL_CHANGE</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>export-excel</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>legacy.demo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
research: portfolio 20261031T145213365962Z-351ea3d6 [NO_MATERIAL_CHANGE]
Imported from local commit 727f39c13363c24dab1f46d1bbf30a75cd1fdc17.
</commit_message>
<xml_diff>
--- a/workbooks/Investment_Workspace.xlsx
+++ b/workbooks/Investment_Workspace.xlsx
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:N10" headerRowCount="1">
-  <autoFilter ref="A1:N10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_Usage" displayName="T_Usage" ref="A1:N11" headerRowCount="1">
+  <autoFilter ref="A1:N11"/>
   <tableColumns count="14">
     <tableColumn id="1" name="cached_input_tokens"/>
     <tableColumn id="2" name="calculation_runtime_seconds"/>
@@ -442,8 +442,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:J10" headerRowCount="1">
-  <autoFilter ref="A1:J10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Run_Log" displayName="T_Run_Log" ref="A1:J11" headerRowCount="1">
+  <autoFilter ref="A1:J11"/>
   <tableColumns count="10">
     <tableColumn id="1" name="analysis_run_id"/>
     <tableColumn id="2" name="attempted_at"/>
@@ -828,7 +828,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20261031T085618170933Z-fbe64605</t>
+          <t>20261031T145213365962Z-351ea3d6</t>
         </is>
       </c>
     </row>
@@ -1958,7 +1958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2644,6 +2644,68 @@
       <c r="N10" t="inlineStr">
         <is>
           <t>{"integration": 4e-06, "portfolio": 0.000417, "valuation": 9e-06, "wealth": 2e-06}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.06574000000000001</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>20261031T145213365962Z-351ea3d6</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>AI telemetry unknown; total wall time recorded externally after commit</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>{"integration": 4e-06, "portfolio": 0.000325, "valuation": 9e-06, "wealth": 2e-06}</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6739,6 +6801,56 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>20261026T225805178235Z-8f6aa76b</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-31T14:52:13.431544+00:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>f7e46148c5af19d0e06edcfffe6b661e851d33406278545dc24ef9487cf65892</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LOCAL_ONLY</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>20261031T145213365962Z-351ea3d6</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>NO_MATERIAL_CHANGE</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>export-excel</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>legacy.demo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>